<commit_message>
fixed structural errors in templates
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionResults/Score-A4.xlsx
+++ b/owlcms/src/main/resources/templates/competitionResults/Score-A4.xlsx
@@ -376,7 +376,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" ns1:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0;;"/>
     <numFmt numFmtId="165" formatCode="_ * #,##0_)\ _$_ ;_ * \(#,##0&quot;) &quot;_$_ ;_ * \-??_)\ _$_ ;_ @_ "/>
@@ -385,7 +385,7 @@
     <numFmt numFmtId="168" formatCode="0.000;;\-"/>
     <numFmt numFmtId="169" formatCode="0;\-;\-"/>
   </numFmts>
-  <fonts count="133" ns2:knownFonts="1">
+  <fonts count="133" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1568,358 +1568,358 @@
       <left/>
       <right/>
       <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -1927,8 +1927,8 @@
       <top style="thin">
         <color indexed="8"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -1936,8 +1936,8 @@
       <top style="thin">
         <color indexed="8"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -1945,50 +1945,50 @@
       <top style="thin">
         <color indexed="8"/>
       </top>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -1996,8 +1996,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2005,8 +2005,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2014,8 +2014,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2023,8 +2023,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2032,8 +2032,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2041,8 +2041,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2050,8 +2050,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2059,8 +2059,8 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left/>
@@ -2068,134 +2068,134 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <diagonal/>
-      <bottom/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="19">
@@ -2585,16 +2585,16 @@
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
     </xf>
     <xf numFmtId="49" fontId="54" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1" applyAlignment="1">
-      <protection locked="0"/>
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="55" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1" applyAlignment="1">
-      <protection locked="0"/>
       <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="56" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1" applyAlignment="1">
-      <protection locked="0"/>
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="0"/>
@@ -2744,16 +2744,16 @@
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
     </xf>
     <xf numFmtId="0" fontId="105" fillId="0" borderId="98" xfId="0" applyProtection="1" applyAlignment="1">
-      <protection locked="0"/>
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="106" fillId="0" borderId="99" xfId="0" applyProtection="1" applyAlignment="1">
-      <protection locked="0"/>
       <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="107" fillId="0" borderId="100" xfId="0" applyProtection="1" applyAlignment="1">
-      <protection locked="0"/>
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="1" fontId="108" fillId="0" borderId="101" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="0"/>
@@ -2793,8 +2793,8 @@
       <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="0"/>
     </xf>
     <xf numFmtId="49" fontId="119" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="0" applyProtection="1" applyAlignment="1" applyFont="1">
-      <protection locked="0"/>
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="120" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyBorder="0">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
@@ -2810,8 +2810,8 @@
       <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="0"/>
     </xf>
     <xf numFmtId="0" fontId="124" fillId="0" borderId="0" xfId="0" applyProtection="1" applyAlignment="1" applyFont="1" applyBorder="0">
-      <protection locked="0"/>
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="125" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="0"/>
@@ -2821,8 +2821,8 @@
       <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="0"/>
     </xf>
     <xf numFmtId="49" fontId="127" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="0" applyProtection="1" applyAlignment="1" applyFont="1">
-      <protection locked="0"/>
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="128" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyFont="1" applyBorder="0">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
@@ -2838,8 +2838,8 @@
       <alignment horizontal="right" vertical="center" wrapText="1" shrinkToFit="0"/>
     </xf>
     <xf numFmtId="0" fontId="132" fillId="0" borderId="0" xfId="0" applyProtection="1" applyAlignment="1" applyFont="1" applyBorder="0">
-      <protection locked="0"/>
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="0"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -2849,18 +2849,18 @@
     <cellStyle name="Accent4" xfId="4" builtinId="41" customBuiltin="1"/>
     <cellStyle name="Accent5" xfId="5" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Accent6" xfId="6" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Emphase 1" xfId="7" ns3:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Emphase 2" xfId="8" ns3:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Emphase 3" xfId="9" ns3:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Emphase 1" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Emphase 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Emphase 3" xfId="9" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="Hyperlink" xfId="10" builtinId="8"/>
-    <cellStyle name="Lien hypertexte 2" xfId="11" ns3:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Lien hypertexte 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="12" ns3:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="Normal 3" xfId="13" ns3:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="Titre 1" xfId="14" ns3:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="Titre 1 1" xfId="15" ns3:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="Titre 1 1 1" xfId="16" ns3:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="Titre de la feuille" xfId="17" ns3:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Normal 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Normal 3" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Titre 1" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Titre 1 1" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Titre 1 1 1" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Titre de la feuille" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Total" xfId="18" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="3">
@@ -2960,10 +2960,10 @@
   </colors>
   <extLst>
     <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <ns4:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
     <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <ns5:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -3316,12 +3316,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Feuil4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:X116"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.85546875" customWidth="1"/>
     <col min="2" max="2" width="5.42578125" style="1" customWidth="1"/>
@@ -3346,14 +3346,14 @@
     <col min="25" max="25" width="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="24" customHeight="1" ns3:dyDescent="0.25">
+    <row r="1" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="199" t="inlineStr">
         <is>
           <t>${competition.competitionName}</t>
         </is>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="24" customHeight="1" ns3:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="200" t="inlineStr">
         <is>
           <t>${t.get("Competition.competitionSite")} :</t>
@@ -3375,7 +3375,7 @@
         </is>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="24" customHeight="1" ns3:dyDescent="0.25">
+    <row r="3" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="200" t="inlineStr">
         <is>
           <t>${t.get("Competition.competitionDate")} :</t>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="24" customHeight="1" ns3:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="205" t="inlineStr">
         <is>
           <t>${session != null ? t.get("Group") + " :" : ""}</t>
@@ -3409,8 +3409,8 @@
         </is>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="6" customHeight="1" ns3:dyDescent="0.2"/>
-    <row r="6" spans="1:24" ht="15" customHeight="1" ns3:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7"/>
       <c r="C6" s="8"/>
       <c r="H6" s="7"/>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="X6"/>
     </row>
-    <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.2">
+    <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>39</v>
       </c>
@@ -3504,7 +3504,7 @@
       <c r="U7" s="99"/>
       <c r="V7" s="101"/>
     </row>
-    <row r="8" spans="1:24" s="19" customFormat="1" ht="7.5" customHeight="1" ns3:dyDescent="0.2">
+    <row r="8" spans="1:24" s="19" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="49"/>
       <c r="B8" s="49"/>
       <c r="C8" s="49"/>
@@ -3518,7 +3518,7 @@
       <c r="K8" s="51"/>
       <c r="V8" s="79"/>
     </row>
-    <row r="9" spans="1:24" ht="21.75" customHeight="1" ns3:dyDescent="0.2">
+    <row r="9" spans="1:24" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="52" t="s">
         <v>47</v>
       </c>
@@ -3547,7 +3547,7 @@
       <c r="V9" s="103"/>
       <c r="X9"/>
     </row>
-    <row r="10" spans="1:24" s="19" customFormat="1" ht="21.2" customHeight="1" ns3:dyDescent="0.2">
+    <row r="10" spans="1:24" s="19" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
         <v>1</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="24.75" customHeight="1" ns3:dyDescent="0.2">
+    <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11"/>
       <c r="G11"/>
       <c r="H11"/>
@@ -3631,14 +3631,14 @@
       <c r="W11"/>
       <c r="X11"/>
     </row>
-    <row r="12" spans="1:24" s="31" customFormat="1" ht="15" ns3:dyDescent="0.25">
+    <row r="12" spans="1:24" s="31" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>56</v>
       </c>
       <c r="J12" s="32"/>
       <c r="V12" s="83"/>
     </row>
-    <row r="13" spans="1:24" s="31" customFormat="1" ht="6.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="13" spans="1:24" s="31" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="56"/>
       <c r="B13" s="56"/>
       <c r="C13" s="56"/>
@@ -3662,7 +3662,7 @@
       <c r="U13" s="62"/>
       <c r="V13" s="84"/>
     </row>
-    <row r="14" spans="1:24" s="74" customFormat="1" ht="12" ns3:dyDescent="0.2">
+    <row r="14" spans="1:24" s="74" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="65" t="s">
         <v>63</v>
       </c>
@@ -3709,7 +3709,7 @@
       <c r="V14" s="85"/>
       <c r="X14" s="67"/>
     </row>
-    <row r="15" spans="1:24" s="55" customFormat="1" ns3:dyDescent="0.2">
+    <row r="15" spans="1:24" s="55" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="57" t="s">
         <v>49</v>
       </c>
@@ -3756,7 +3756,7 @@
       <c r="V15" s="86"/>
       <c r="X15" s="59"/>
     </row>
-    <row r="16" spans="1:24" ns3:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="H16" s="2"/>
@@ -3768,314 +3768,314 @@
       <c r="S16" s="1"/>
       <c r="T16" s="12"/>
     </row>
-    <row r="17" spans="4:21" ns3:dyDescent="0.2">
+    <row r="17" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F17" s="1"/>
       <c r="U17" s="12"/>
     </row>
-    <row r="18" spans="4:21" ns3:dyDescent="0.2">
+    <row r="18" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F18" s="1"/>
       <c r="U18" s="12"/>
     </row>
-    <row r="19" spans="4:21" ns3:dyDescent="0.2">
+    <row r="19" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F19" s="1"/>
       <c r="U19" s="12"/>
     </row>
-    <row r="20" spans="4:21" ns3:dyDescent="0.2">
+    <row r="20" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F20" s="1"/>
       <c r="U20" s="12"/>
     </row>
-    <row r="21" spans="4:21" ns3:dyDescent="0.2">
+    <row r="21" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F21" s="1"/>
       <c r="U21" s="12"/>
     </row>
-    <row r="22" spans="4:21" ns3:dyDescent="0.2">
+    <row r="22" spans="4:21" x14ac:dyDescent="0.2">
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="1"/>
       <c r="U22" s="12"/>
     </row>
-    <row r="23" spans="4:21" ns3:dyDescent="0.2">
+    <row r="23" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F23" s="1"/>
       <c r="U23" s="12"/>
     </row>
-    <row r="24" spans="4:21" ns3:dyDescent="0.2">
+    <row r="24" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F24" s="1"/>
       <c r="U24" s="12"/>
     </row>
-    <row r="25" spans="4:21" ns3:dyDescent="0.2">
+    <row r="25" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="4:21" ns3:dyDescent="0.2">
+    <row r="26" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="4:21" ns3:dyDescent="0.2">
+    <row r="27" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="4:21" ns3:dyDescent="0.2">
+    <row r="28" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="4:21" ns3:dyDescent="0.2">
+    <row r="29" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="4:21" ns3:dyDescent="0.2">
+    <row r="30" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F30" s="1"/>
     </row>
-    <row r="31" spans="4:21" ns3:dyDescent="0.2">
+    <row r="31" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F31" s="1"/>
     </row>
-    <row r="32" spans="4:21" ns3:dyDescent="0.2">
+    <row r="32" spans="4:21" x14ac:dyDescent="0.2">
       <c r="F32" s="1"/>
     </row>
-    <row r="33" spans="6:6" ns3:dyDescent="0.2">
+    <row r="33" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F33" s="1"/>
     </row>
-    <row r="34" spans="6:6" ns3:dyDescent="0.2">
+    <row r="34" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F34" s="1"/>
     </row>
-    <row r="35" spans="6:6" ns3:dyDescent="0.2">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="6:6" ns3:dyDescent="0.2">
+    <row r="36" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F36" s="1"/>
     </row>
-    <row r="37" spans="6:6" ns3:dyDescent="0.2">
+    <row r="37" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F37" s="1"/>
     </row>
-    <row r="38" spans="6:6" ns3:dyDescent="0.2">
+    <row r="38" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F38" s="1"/>
     </row>
-    <row r="39" spans="6:6" ns3:dyDescent="0.2">
+    <row r="39" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F39" s="1"/>
     </row>
-    <row r="40" spans="6:6" ns3:dyDescent="0.2">
+    <row r="40" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F40" s="1"/>
     </row>
-    <row r="41" spans="6:6" ns3:dyDescent="0.2">
+    <row r="41" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F41" s="1"/>
     </row>
-    <row r="42" spans="6:6" ns3:dyDescent="0.2">
+    <row r="42" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F42" s="1"/>
     </row>
-    <row r="43" spans="6:6" ns3:dyDescent="0.2">
+    <row r="43" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F43" s="1"/>
     </row>
-    <row r="44" spans="6:6" ns3:dyDescent="0.2">
+    <row r="44" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F44" s="1"/>
     </row>
-    <row r="45" spans="6:6" ns3:dyDescent="0.2">
+    <row r="45" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F45" s="1"/>
     </row>
-    <row r="46" spans="6:6" ns3:dyDescent="0.2">
+    <row r="46" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F46" s="1"/>
     </row>
-    <row r="47" spans="6:6" ns3:dyDescent="0.2">
+    <row r="47" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F47" s="1"/>
     </row>
-    <row r="48" spans="6:6" ns3:dyDescent="0.2">
+    <row r="48" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F48" s="1"/>
     </row>
-    <row r="49" spans="6:6" ns3:dyDescent="0.2">
+    <row r="49" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F49" s="1"/>
     </row>
-    <row r="50" spans="6:6" ns3:dyDescent="0.2">
+    <row r="50" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F50" s="1"/>
     </row>
-    <row r="51" spans="6:6" ns3:dyDescent="0.2">
+    <row r="51" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F51" s="1"/>
     </row>
-    <row r="52" spans="6:6" ns3:dyDescent="0.2">
+    <row r="52" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F52" s="1"/>
     </row>
-    <row r="53" spans="6:6" ns3:dyDescent="0.2">
+    <row r="53" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F53" s="1"/>
     </row>
-    <row r="54" spans="6:6" ns3:dyDescent="0.2">
+    <row r="54" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F54" s="1"/>
     </row>
-    <row r="55" spans="6:6" ns3:dyDescent="0.2">
+    <row r="55" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F55" s="1"/>
     </row>
-    <row r="56" spans="6:6" ns3:dyDescent="0.2">
+    <row r="56" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F56" s="1"/>
     </row>
-    <row r="57" spans="6:6" ns3:dyDescent="0.2">
+    <row r="57" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F57" s="1"/>
     </row>
-    <row r="58" spans="6:6" ns3:dyDescent="0.2">
+    <row r="58" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F58" s="1"/>
     </row>
-    <row r="59" spans="6:6" ns3:dyDescent="0.2">
+    <row r="59" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F59" s="1"/>
     </row>
-    <row r="60" spans="6:6" ns3:dyDescent="0.2">
+    <row r="60" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F60" s="1"/>
     </row>
-    <row r="61" spans="6:6" ns3:dyDescent="0.2">
+    <row r="61" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F61" s="1"/>
     </row>
-    <row r="62" spans="6:6" ns3:dyDescent="0.2">
+    <row r="62" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F62" s="1"/>
     </row>
-    <row r="63" spans="6:6" ns3:dyDescent="0.2">
+    <row r="63" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F63" s="1"/>
     </row>
-    <row r="64" spans="6:6" ns3:dyDescent="0.2">
+    <row r="64" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F64" s="1"/>
     </row>
-    <row r="65" spans="6:6" ns3:dyDescent="0.2">
+    <row r="65" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F65" s="1"/>
     </row>
-    <row r="66" spans="6:6" ns3:dyDescent="0.2">
+    <row r="66" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F66" s="1"/>
     </row>
-    <row r="67" spans="6:6" ns3:dyDescent="0.2">
+    <row r="67" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F67" s="1"/>
     </row>
-    <row r="68" spans="6:6" ns3:dyDescent="0.2">
+    <row r="68" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F68" s="1"/>
     </row>
-    <row r="69" spans="6:6" ns3:dyDescent="0.2">
+    <row r="69" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F69" s="1"/>
     </row>
-    <row r="70" spans="6:6" ns3:dyDescent="0.2">
+    <row r="70" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F70" s="1"/>
     </row>
-    <row r="71" spans="6:6" ns3:dyDescent="0.2">
+    <row r="71" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F71" s="1"/>
     </row>
-    <row r="72" spans="6:6" ns3:dyDescent="0.2">
+    <row r="72" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F72" s="1"/>
     </row>
-    <row r="73" spans="6:6" ns3:dyDescent="0.2">
+    <row r="73" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F73" s="1"/>
     </row>
-    <row r="74" spans="6:6" ns3:dyDescent="0.2">
+    <row r="74" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F74" s="1"/>
     </row>
-    <row r="75" spans="6:6" ns3:dyDescent="0.2">
+    <row r="75" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F75" s="1"/>
     </row>
-    <row r="76" spans="6:6" ns3:dyDescent="0.2">
+    <row r="76" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F76" s="1"/>
     </row>
-    <row r="77" spans="6:6" ns3:dyDescent="0.2">
+    <row r="77" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F77" s="1"/>
     </row>
-    <row r="78" spans="6:6" ns3:dyDescent="0.2">
+    <row r="78" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F78" s="1"/>
     </row>
-    <row r="79" spans="6:6" ns3:dyDescent="0.2">
+    <row r="79" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F79" s="1"/>
     </row>
-    <row r="80" spans="6:6" ns3:dyDescent="0.2">
+    <row r="80" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F80" s="1"/>
     </row>
-    <row r="81" spans="6:6" ns3:dyDescent="0.2">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F81" s="1"/>
     </row>
-    <row r="82" spans="6:6" ns3:dyDescent="0.2">
+    <row r="82" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F82" s="1"/>
     </row>
-    <row r="83" spans="6:6" ns3:dyDescent="0.2">
+    <row r="83" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F83" s="1"/>
     </row>
-    <row r="84" spans="6:6" ns3:dyDescent="0.2">
+    <row r="84" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F84" s="1"/>
     </row>
-    <row r="85" spans="6:6" ns3:dyDescent="0.2">
+    <row r="85" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F85" s="1"/>
     </row>
-    <row r="86" spans="6:6" ns3:dyDescent="0.2">
+    <row r="86" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F86" s="1"/>
     </row>
-    <row r="87" spans="6:6" ns3:dyDescent="0.2">
+    <row r="87" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F87" s="1"/>
     </row>
-    <row r="88" spans="6:6" ns3:dyDescent="0.2">
+    <row r="88" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F88" s="1"/>
     </row>
-    <row r="89" spans="6:6" ns3:dyDescent="0.2">
+    <row r="89" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F89" s="1"/>
     </row>
-    <row r="90" spans="6:6" ns3:dyDescent="0.2">
+    <row r="90" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F90" s="1"/>
     </row>
-    <row r="91" spans="6:6" ns3:dyDescent="0.2">
+    <row r="91" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F91" s="1"/>
     </row>
-    <row r="92" spans="6:6" ns3:dyDescent="0.2">
+    <row r="92" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F92" s="1"/>
     </row>
-    <row r="93" spans="6:6" ns3:dyDescent="0.2">
+    <row r="93" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F93" s="1"/>
     </row>
-    <row r="94" spans="6:6" ns3:dyDescent="0.2">
+    <row r="94" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F94" s="1"/>
     </row>
-    <row r="95" spans="6:6" ns3:dyDescent="0.2">
+    <row r="95" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F95" s="1"/>
     </row>
-    <row r="96" spans="6:6" ns3:dyDescent="0.2">
+    <row r="96" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F96" s="1"/>
     </row>
-    <row r="97" spans="6:6" ns3:dyDescent="0.2">
+    <row r="97" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F97" s="1"/>
     </row>
-    <row r="98" spans="6:6" ns3:dyDescent="0.2">
+    <row r="98" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F98" s="1"/>
     </row>
-    <row r="99" spans="6:6" ns3:dyDescent="0.2">
+    <row r="99" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F99" s="1"/>
     </row>
-    <row r="100" spans="6:6" ns3:dyDescent="0.2">
+    <row r="100" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F100" s="1"/>
     </row>
-    <row r="101" spans="6:6" ns3:dyDescent="0.2">
+    <row r="101" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F101" s="1"/>
     </row>
-    <row r="102" spans="6:6" ns3:dyDescent="0.2">
+    <row r="102" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F102" s="1"/>
     </row>
-    <row r="103" spans="6:6" ns3:dyDescent="0.2">
+    <row r="103" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F103" s="1"/>
     </row>
-    <row r="104" spans="6:6" ns3:dyDescent="0.2">
+    <row r="104" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F104" s="1"/>
     </row>
-    <row r="105" spans="6:6" ns3:dyDescent="0.2">
+    <row r="105" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F105" s="1"/>
     </row>
-    <row r="106" spans="6:6" ns3:dyDescent="0.2">
+    <row r="106" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F106" s="1"/>
     </row>
-    <row r="107" spans="6:6" ns3:dyDescent="0.2">
+    <row r="107" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F107" s="1"/>
     </row>
-    <row r="108" spans="6:6" ns3:dyDescent="0.2">
+    <row r="108" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F108" s="1"/>
     </row>
-    <row r="109" spans="6:6" ns3:dyDescent="0.2">
+    <row r="109" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F109" s="1"/>
     </row>
-    <row r="110" spans="6:6" ns3:dyDescent="0.2">
+    <row r="110" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F110" s="1"/>
     </row>
-    <row r="111" spans="6:6" ns3:dyDescent="0.2">
+    <row r="111" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F111" s="1"/>
     </row>
-    <row r="112" spans="6:6" ns3:dyDescent="0.2">
+    <row r="112" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F112" s="1"/>
     </row>
-    <row r="113" spans="6:6" ns3:dyDescent="0.2">
+    <row r="113" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F113" s="1"/>
     </row>
-    <row r="114" spans="6:6" ns3:dyDescent="0.2">
+    <row r="114" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F114" s="1"/>
     </row>
-    <row r="115" spans="6:6" ns3:dyDescent="0.2">
+    <row r="115" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F115" s="1"/>
     </row>
-    <row r="116" spans="6:6" ns3:dyDescent="0.2">
+    <row r="116" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F116" s="1"/>
     </row>
   </sheetData>
@@ -4102,37 +4102,21 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="D4:V4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C8:D8">
-    <cfRule type="expression" dxfId="2" priority="7" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D10:E10">
-    <cfRule type="expression" dxfId="1" priority="11" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D11:F13">
-    <cfRule type="expression" dxfId="0" priority="5" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation showErrorMessage="1" sqref="K4" ns2:uid="{00000000-0002-0000-0000-000000000000}"/>
-    <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" ns2:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="H11:H13" ns2:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation showErrorMessage="1" sqref="K4" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" sqref="H10" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="H11:H13" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I8" ns2:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I8" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
   </dataValidations>
-  <hyperlinks/>
   <pageMargins left="0.31496062992125984" right="0.35433070866141736" top="0.39370078740157483" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="70" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" ns4:id="rId3"/>
+  <pageSetup paperSize="9" scale="70" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
   <headerFooter alignWithMargins="0"/>
-  <legacyDrawing ns4:id="rId4"/>
+  <legacyDrawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>